<commit_message>
Added support for dollars in AmericanUnits
</commit_message>
<xml_diff>
--- a/assets/code-files/american-units/UnitsSources.xlsx
+++ b/assets/code-files/american-units/UnitsSources.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="265">
   <si>
     <t>Unit Name</t>
   </si>
@@ -619,6 +619,66 @@
     <t>https://www.cradleofaviation.org/history/history/saturn-v-rocket.html</t>
   </si>
   <si>
+    <t>Pressure of a US dollar bill lying flat</t>
+  </si>
+  <si>
+    <t>pascals</t>
+  </si>
+  <si>
+    <t>https://web.archive.org/web/20060906152305/http://www.dac.neu.edu/physics/b.maheswaran/phy1222/fluids.pdf</t>
+  </si>
+  <si>
+    <t>Pressure of a penny</t>
+  </si>
+  <si>
+    <t>https://physics.stackexchange.com/questions/12191/get-an-intuition-for-pressure-values/12252#12252</t>
+  </si>
+  <si>
+    <t>Pressure of a quarter</t>
+  </si>
+  <si>
+    <t>https://web.archive.org/web/20150218061037/http://www.usmint.gov/about_the_mint/?action=coin_specifications</t>
+  </si>
+  <si>
+    <t>Gauge Pressure of Ford F-150 tire</t>
+  </si>
+  <si>
+    <t>https://www.riversideford.net/blog/what-tire-psi-is-recommended-on-the-ford-f-150/</t>
+  </si>
+  <si>
+    <t>Maximum pressure for an attack submarine</t>
+  </si>
+  <si>
+    <t>https://www.usamm.com/blogs/news/how-deep-can-a-navy-submarine-go</t>
+  </si>
+  <si>
+    <t>Overpressure of Oklahoma City bombing</t>
+  </si>
+  <si>
+    <t>https://www.industrytap.com/bomb-proof-concrete-wallpaper-designed-to-save-lives/4518</t>
+  </si>
+  <si>
+    <t>Pressure inside barrel of a .50 caliber firearm when firing</t>
+  </si>
+  <si>
+    <t>https://cuttingedgebullets.com/blogs/news/the-historical-future-of-the-50bmg</t>
+  </si>
+  <si>
+    <t>Pressure generated by the National Ignition Facility's Fusion Reactor</t>
+  </si>
+  <si>
+    <t>https://str.llnl.gov/past-issues/september-2019/gently-compressing-materials-record-levels</t>
+  </si>
+  <si>
+    <t>Pressure generated by Ivy Mike Hydrogen Bomb</t>
+  </si>
+  <si>
+    <t>https://nuclearweaponarchive.org/Nwfaq/Nfaq4-4.html#Nfaq4.4.3.3</t>
+  </si>
+  <si>
+    <t>Pressure generated by W80 Hydrogen Bomb</t>
+  </si>
+  <si>
     <t>Time it takes for one step of a nuclear chain reaction</t>
   </si>
   <si>
@@ -813,6 +873,54 @@
   </si>
   <si>
     <t>https://www.lle.rochester.edu/omega-laser-facility/omega-ep/</t>
+  </si>
+  <si>
+    <t>One year of U.S. Military</t>
+  </si>
+  <si>
+    <t>dollars</t>
+  </si>
+  <si>
+    <t>https://www.macrotrends.net/global-metrics/countries/usa/united-states/military-spending-defense-budget</t>
+  </si>
+  <si>
+    <t>One month of U.S. Military</t>
+  </si>
+  <si>
+    <t>One day of U.S. Military</t>
+  </si>
+  <si>
+    <t>One hour of U.S. Military</t>
+  </si>
+  <si>
+    <t>One minute of U.S. Military</t>
+  </si>
+  <si>
+    <t>One second of U.S. Military</t>
+  </si>
+  <si>
+    <t>Average American Healthcare Spending in a Year</t>
+  </si>
+  <si>
+    <t>https://www.cms.gov/data-research/statistics-trends-and-reports/national-health-expenditure-data/historical</t>
+  </si>
+  <si>
+    <t>Average college tuition in the U.S.</t>
+  </si>
+  <si>
+    <t>https://educationdata.org/average-cost-of-college</t>
+  </si>
+  <si>
+    <t>Cost to see MLB baseball game</t>
+  </si>
+  <si>
+    <t>https://www.nytimes.com/athletic/2830372/2021/09/16/what-it-costs-for-every-mlb-teams-fans-to-attend-a-game-and-why-the-average-price-went-up-in-2021/</t>
+  </si>
+  <si>
+    <t>Cost of a Costco Hot Dog</t>
+  </si>
+  <si>
+    <t>https://www.rd.com/article/reason-costco-hot-dogs-cheap/</t>
   </si>
 </sst>
 </file>
@@ -871,7 +979,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -886,7 +994,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -2646,13 +2754,12 @@
       <c r="B81" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C81" s="8">
-        <f>10^-8</f>
-        <v>0.00000001</v>
+      <c r="C81" s="3">
+        <v>1.0</v>
       </c>
       <c r="D81" s="4">
         <f t="shared" si="1"/>
-        <v>100000000</v>
+        <v>1</v>
       </c>
       <c r="E81" s="5" t="s">
         <v>166</v>
@@ -2666,12 +2773,11 @@
         <v>165</v>
       </c>
       <c r="C82" s="3">
-        <f>1/100</f>
-        <v>0.01</v>
+        <v>86.0</v>
       </c>
       <c r="D82" s="4">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>0.01162790698</v>
       </c>
       <c r="E82" s="5" t="s">
         <v>168</v>
@@ -2684,13 +2790,12 @@
       <c r="B83" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C83" s="8">
-        <f>1/3</f>
-        <v>0.3333333333</v>
+      <c r="C83" s="3">
+        <v>120.0</v>
       </c>
       <c r="D83" s="4">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>0.008333333333</v>
       </c>
       <c r="E83" s="5" t="s">
         <v>170</v>
@@ -2704,13 +2809,13 @@
         <v>165</v>
       </c>
       <c r="C84" s="3">
-        <v>10.0</v>
+        <v>258553.4</v>
       </c>
       <c r="D84" s="4">
         <f t="shared" si="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="E84" s="9" t="s">
+        <v>0.000003867672984</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>172</v>
       </c>
     </row>
@@ -2722,11 +2827,11 @@
         <v>165</v>
       </c>
       <c r="C85" s="3">
-        <v>103.0</v>
+        <v>2384190.0</v>
       </c>
       <c r="D85" s="4">
         <f t="shared" si="1"/>
-        <v>0.009708737864</v>
+        <v>0.0000004194296595</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>174</v>
@@ -2740,11 +2845,11 @@
         <v>165</v>
       </c>
       <c r="C86" s="3">
-        <v>1200.0</v>
+        <v>2.8E7</v>
       </c>
       <c r="D86" s="4">
         <f t="shared" si="1"/>
-        <v>0.0008333333333</v>
+        <v>0.00000003571428571</v>
       </c>
       <c r="E86" s="5" t="s">
         <v>176</v>
@@ -2758,11 +2863,11 @@
         <v>165</v>
       </c>
       <c r="C87" s="3">
-        <v>12600.0</v>
+        <v>4.82633E8</v>
       </c>
       <c r="D87" s="4">
         <f t="shared" si="1"/>
-        <v>0.00007936507937</v>
+        <v>0.000000002071967727</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>178</v>
@@ -2776,11 +2881,11 @@
         <v>165</v>
       </c>
       <c r="C88" s="3">
-        <v>154440.0</v>
+        <v>5.0E12</v>
       </c>
       <c r="D88" s="4">
         <f t="shared" si="1"/>
-        <v>0.000006475006475</v>
+        <v>0</v>
       </c>
       <c r="E88" s="5" t="s">
         <v>180</v>
@@ -2794,11 +2899,11 @@
         <v>165</v>
       </c>
       <c r="C89" s="3">
-        <v>2637000.0</v>
+        <v>5.4E14</v>
       </c>
       <c r="D89" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000003792188093</v>
+        <v>0</v>
       </c>
       <c r="E89" s="5" t="s">
         <v>182</v>
@@ -2812,29 +2917,30 @@
         <v>165</v>
       </c>
       <c r="C90" s="3">
-        <v>1.823E7</v>
+        <v>6.5E15</v>
       </c>
       <c r="D90" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000005485463522</v>
+        <v>0</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="91" ht="22.5" customHeight="1">
       <c r="A91" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B91" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="B91" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C91" s="3">
-        <v>6.312E7</v>
+      <c r="C91" s="8">
+        <f>10^-8</f>
+        <v>0.00000001</v>
       </c>
       <c r="D91" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000001584283904</v>
+        <v>100000000</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>186</v>
@@ -2845,122 +2951,124 @@
         <v>187</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="C92" s="3">
-        <v>1.893E8</v>
+        <f>1/100</f>
+        <v>0.01</v>
       </c>
       <c r="D92" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000000528262018</v>
+        <v>100</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="93" ht="22.5" customHeight="1">
       <c r="A93" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C93" s="3">
-        <v>2.0123E8</v>
+        <v>185</v>
+      </c>
+      <c r="C93" s="8">
+        <f>1/3</f>
+        <v>0.3333333333</v>
       </c>
       <c r="D93" s="4">
         <f t="shared" si="1"/>
-        <v>0.000000004969437957</v>
+        <v>3</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="94" ht="22.5" customHeight="1">
       <c r="A94" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="C94" s="3">
-        <v>7.88728E9</v>
+        <v>10.0</v>
       </c>
       <c r="D94" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000000001267864207</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>191</v>
+        <v>0.1</v>
+      </c>
+      <c r="E94" s="9" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="95" ht="22.5" customHeight="1">
       <c r="A95" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="C95" s="3">
-        <v>1.684092E10</v>
+        <v>103.0</v>
       </c>
       <c r="D95" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.009708737864</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="96" ht="22.5" customHeight="1">
       <c r="A96" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="C96" s="3">
-        <v>9.4608E11</v>
+        <v>1200.0</v>
       </c>
       <c r="D96" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.0008333333333</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="97" ht="22.5" customHeight="1">
       <c r="A97" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="C97" s="3">
-        <v>1.0233782E15</v>
+        <v>12600.0</v>
       </c>
       <c r="D97" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E97" s="9" t="s">
-        <v>197</v>
+        <v>0.00007936507937</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="98" ht="22.5" customHeight="1">
       <c r="A98" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="C98" s="3">
-        <v>50.0</v>
+        <v>154440.0</v>
       </c>
       <c r="D98" s="4">
         <f t="shared" si="1"/>
-        <v>0.02</v>
+        <v>0.000006475006475</v>
       </c>
       <c r="E98" s="5" t="s">
         <v>200</v>
@@ -2971,14 +3079,14 @@
         <v>201</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="C99" s="3">
-        <v>60.0</v>
+        <v>2637000.0</v>
       </c>
       <c r="D99" s="4">
         <f t="shared" si="1"/>
-        <v>0.01666666667</v>
+        <v>0.0000003792188093</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>202</v>
@@ -2989,32 +3097,32 @@
         <v>203</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="C100" s="3">
-        <v>9334.11285138</v>
+        <v>1.823E7</v>
       </c>
       <c r="D100" s="4">
         <f t="shared" si="1"/>
-        <v>0.0001071339093</v>
+        <v>0.00000005485463522</v>
       </c>
       <c r="E100" s="5" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="101" ht="22.5" customHeight="1">
-      <c r="A101" s="7" t="s">
+      <c r="A101" s="1" t="s">
         <v>205</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="C101" s="3">
-        <v>100000.0</v>
+        <v>6.312E7</v>
       </c>
       <c r="D101" s="4">
         <f t="shared" si="1"/>
-        <v>0.00001</v>
+        <v>0.00000001584283904</v>
       </c>
       <c r="E101" s="5" t="s">
         <v>206</v>
@@ -3025,122 +3133,122 @@
         <v>207</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="C102" s="3">
-        <v>514849.0</v>
+        <v>1.893E8</v>
       </c>
       <c r="D102" s="4">
         <f t="shared" si="1"/>
-        <v>0.000001942317068</v>
+        <v>0.00000000528262018</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="103" ht="22.5" customHeight="1">
       <c r="A103" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C103" s="3">
+        <v>2.0123E8</v>
+      </c>
+      <c r="D103" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000004969437957</v>
+      </c>
+      <c r="E103" s="5" t="s">
         <v>209</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C103" s="3">
-        <v>1265058.0</v>
-      </c>
-      <c r="D103" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000007904775908</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="104" ht="22.5" customHeight="1">
       <c r="A104" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C104" s="3">
+        <v>7.88728E9</v>
+      </c>
+      <c r="D104" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000000001267864207</v>
+      </c>
+      <c r="E104" s="5" t="s">
         <v>211</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C104" s="3">
-        <v>2.5742456E7</v>
-      </c>
-      <c r="D104" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000000388463323</v>
-      </c>
-      <c r="E104" s="5" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="105" ht="22.5" customHeight="1">
       <c r="A105" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C105" s="3">
+        <v>1.684092E10</v>
+      </c>
+      <c r="D105" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E105" s="5" t="s">
         <v>213</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C105" s="3">
-        <v>1.91229675E8</v>
-      </c>
-      <c r="D105" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000000005229313913</v>
-      </c>
-      <c r="E105" s="5" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="106" ht="22.5" customHeight="1">
       <c r="A106" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C106" s="3">
+        <v>9.4608E11</v>
+      </c>
+      <c r="D106" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E106" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C106" s="3">
-        <v>2.08E9</v>
-      </c>
-      <c r="D106" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000000004807692308</v>
-      </c>
-      <c r="E106" s="5" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="107" ht="22.5" customHeight="1">
       <c r="A107" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C107" s="3">
+        <v>1.0233782E15</v>
+      </c>
+      <c r="D107" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E107" s="9" t="s">
         <v>217</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C107" s="3">
-        <v>1.2E10</v>
-      </c>
-      <c r="D107" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E107" s="5" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="108" ht="22.5" customHeight="1">
       <c r="A108" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B108" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="B108" s="1" t="s">
-        <v>199</v>
-      </c>
       <c r="C108" s="3">
-        <v>8.81529680365E10</v>
+        <v>50.0</v>
       </c>
       <c r="D108" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E108" s="5" t="s">
         <v>220</v>
@@ -3151,16 +3259,16 @@
         <v>221</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="C109" s="3">
-        <v>2.39E11</v>
+        <v>60.0</v>
       </c>
       <c r="D109" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E109" s="9" t="s">
+        <v>0.01666666667</v>
+      </c>
+      <c r="E109" s="5" t="s">
         <v>222</v>
       </c>
     </row>
@@ -3169,33 +3277,32 @@
         <v>223</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="C110" s="3">
-        <v>3.2552635E12</v>
+        <v>9334.11285138</v>
       </c>
       <c r="D110" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.0001071339093</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="111" ht="22.5" customHeight="1">
-      <c r="A111" s="1" t="s">
+      <c r="A111" s="7" t="s">
         <v>225</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C111" s="8">
-        <f>3*10^14</f>
-        <v>300000000000000</v>
+        <v>219</v>
+      </c>
+      <c r="C111" s="3">
+        <v>100000.0</v>
       </c>
       <c r="D111" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.00001</v>
       </c>
       <c r="E111" s="5" t="s">
         <v>226</v>
@@ -3206,223 +3313,384 @@
         <v>227</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="C112" s="3">
-        <v>1.4285714E15</v>
+        <v>514849.0</v>
       </c>
       <c r="D112" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.000001942317068</v>
       </c>
       <c r="E112" s="5" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="113" ht="22.5" customHeight="1">
-      <c r="A113" s="10"/>
-      <c r="B113" s="10"/>
-      <c r="C113" s="8"/>
-      <c r="D113" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E113" s="11"/>
+      <c r="A113" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C113" s="3">
+        <v>1265058.0</v>
+      </c>
+      <c r="D113" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000007904775908</v>
+      </c>
+      <c r="E113" s="5" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="114" ht="22.5" customHeight="1">
-      <c r="A114" s="10"/>
-      <c r="B114" s="10"/>
-      <c r="C114" s="8"/>
-      <c r="D114" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E114" s="11"/>
+      <c r="A114" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C114" s="3">
+        <v>2.5742456E7</v>
+      </c>
+      <c r="D114" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000000388463323</v>
+      </c>
+      <c r="E114" s="5" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="115" ht="22.5" customHeight="1">
-      <c r="A115" s="10"/>
-      <c r="B115" s="10"/>
-      <c r="C115" s="8"/>
-      <c r="D115" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E115" s="11"/>
+      <c r="A115" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C115" s="3">
+        <v>1.91229675E8</v>
+      </c>
+      <c r="D115" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000005229313913</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="116" ht="22.5" customHeight="1">
-      <c r="A116" s="10"/>
-      <c r="B116" s="10"/>
-      <c r="C116" s="8"/>
-      <c r="D116" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E116" s="11"/>
+      <c r="A116" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C116" s="3">
+        <v>2.08E9</v>
+      </c>
+      <c r="D116" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000000004807692308</v>
+      </c>
+      <c r="E116" s="5" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="117" ht="22.5" customHeight="1">
-      <c r="A117" s="10"/>
-      <c r="B117" s="10"/>
-      <c r="C117" s="8"/>
-      <c r="D117" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E117" s="11"/>
+      <c r="A117" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C117" s="3">
+        <v>1.2E10</v>
+      </c>
+      <c r="D117" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E117" s="5" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="118" ht="22.5" customHeight="1">
-      <c r="A118" s="10"/>
-      <c r="B118" s="10"/>
-      <c r="C118" s="8"/>
-      <c r="D118" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E118" s="11"/>
+      <c r="A118" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C118" s="3">
+        <v>8.81529680365E10</v>
+      </c>
+      <c r="D118" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="119" ht="22.5" customHeight="1">
-      <c r="A119" s="10"/>
-      <c r="B119" s="10"/>
-      <c r="C119" s="8"/>
-      <c r="D119" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E119" s="11"/>
+      <c r="A119" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C119" s="3">
+        <v>2.39E11</v>
+      </c>
+      <c r="D119" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E119" s="9" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="120" ht="22.5" customHeight="1">
-      <c r="A120" s="10"/>
-      <c r="B120" s="10"/>
-      <c r="C120" s="8"/>
-      <c r="D120" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E120" s="11"/>
+      <c r="A120" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C120" s="3">
+        <v>3.2552635E12</v>
+      </c>
+      <c r="D120" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="121" ht="22.5" customHeight="1">
-      <c r="A121" s="10"/>
-      <c r="B121" s="10"/>
-      <c r="C121" s="8"/>
-      <c r="D121" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E121" s="11"/>
+      <c r="A121" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C121" s="8">
+        <f>3*10^14</f>
+        <v>300000000000000</v>
+      </c>
+      <c r="D121" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="122" ht="22.5" customHeight="1">
-      <c r="A122" s="10"/>
-      <c r="B122" s="10"/>
-      <c r="C122" s="8"/>
-      <c r="D122" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E122" s="11"/>
+      <c r="A122" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C122" s="3">
+        <v>1.4285714E15</v>
+      </c>
+      <c r="D122" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="123" ht="22.5" customHeight="1">
-      <c r="A123" s="10"/>
-      <c r="B123" s="10"/>
-      <c r="C123" s="8"/>
-      <c r="D123" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E123" s="11"/>
+      <c r="A123" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C123" s="3">
+        <v>9.9731E11</v>
+      </c>
+      <c r="D123" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E123" s="5" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="124" ht="22.5" customHeight="1">
-      <c r="A124" s="10"/>
-      <c r="B124" s="10"/>
-      <c r="C124" s="8"/>
-      <c r="D124" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E124" s="11"/>
+      <c r="A124" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C124" s="3">
+        <v>8.31091666667E10</v>
+      </c>
+      <c r="D124" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E124" s="5" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="125" ht="22.5" customHeight="1">
-      <c r="A125" s="10"/>
-      <c r="B125" s="10"/>
-      <c r="C125" s="8"/>
-      <c r="D125" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E125" s="11"/>
+      <c r="A125" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C125" s="3">
+        <v>2.73235616438E9</v>
+      </c>
+      <c r="D125" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000000003659844983</v>
+      </c>
+      <c r="E125" s="5" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="126" ht="22.5" customHeight="1">
-      <c r="A126" s="10"/>
-      <c r="B126" s="10"/>
-      <c r="C126" s="8"/>
-      <c r="D126" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E126" s="11"/>
+      <c r="A126" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C126" s="3">
+        <v>1.13848173516E8</v>
+      </c>
+      <c r="D126" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000008783627959</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="127" ht="22.5" customHeight="1">
-      <c r="A127" s="10"/>
-      <c r="B127" s="10"/>
-      <c r="C127" s="8"/>
-      <c r="D127" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E127" s="11"/>
+      <c r="A127" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C127" s="3">
+        <v>1897469.5586</v>
+      </c>
+      <c r="D127" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000005270176776</v>
+      </c>
+      <c r="E127" s="5" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="128" ht="22.5" customHeight="1">
-      <c r="A128" s="10"/>
-      <c r="B128" s="10"/>
-      <c r="C128" s="8"/>
-      <c r="D128" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E128" s="11"/>
+      <c r="A128" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C128" s="3">
+        <v>31624.4926433</v>
+      </c>
+      <c r="D128" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00003162106065</v>
+      </c>
+      <c r="E128" s="5" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="129" ht="22.5" customHeight="1">
-      <c r="A129" s="10"/>
-      <c r="B129" s="10"/>
-      <c r="C129" s="8"/>
-      <c r="D129" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E129" s="11"/>
+      <c r="A129" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C129" s="3">
+        <v>15474.0</v>
+      </c>
+      <c r="D129" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00006462453147</v>
+      </c>
+      <c r="E129" s="5" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="130" ht="22.5" customHeight="1">
-      <c r="A130" s="10"/>
-      <c r="B130" s="10"/>
-      <c r="C130" s="8"/>
-      <c r="D130" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E130" s="11"/>
+      <c r="A130" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C130" s="3">
+        <v>38270.0</v>
+      </c>
+      <c r="D130" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00002613012804</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="131" ht="22.5" customHeight="1">
-      <c r="A131" s="10"/>
-      <c r="B131" s="10"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E131" s="11"/>
+      <c r="A131" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C131" s="3">
+        <v>63.25</v>
+      </c>
+      <c r="D131" s="4">
+        <f t="shared" si="1"/>
+        <v>0.01581027668</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>262</v>
+      </c>
     </row>
     <row r="132" ht="22.5" customHeight="1">
-      <c r="A132" s="10"/>
-      <c r="B132" s="10"/>
-      <c r="C132" s="8"/>
-      <c r="D132" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E132" s="11"/>
+      <c r="A132" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C132" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="D132" s="4">
+        <f t="shared" si="1"/>
+        <v>0.6666666667</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>264</v>
+      </c>
     </row>
     <row r="133" ht="22.5" customHeight="1">
       <c r="A133" s="10"/>
       <c r="B133" s="10"/>
-      <c r="C133" s="8"/>
+      <c r="C133" s="3"/>
       <c r="D133" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -12240,6 +12508,11 @@
       <c r="E1014" s="11"/>
     </row>
   </sheetData>
+  <dataValidations>
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="C2:C1014">
+      <formula1>AND(ISNUMBER(C2),(NOT(OR(NOT(ISERROR(DATEVALUE(C2))), AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D")))))</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="E2"/>
     <hyperlink r:id="rId2" ref="E3"/>
@@ -12321,15 +12594,15 @@
     <hyperlink r:id="rId78" ref="E79"/>
     <hyperlink r:id="rId79" ref="E80"/>
     <hyperlink r:id="rId80" ref="E81"/>
-    <hyperlink r:id="rId81" ref="E82"/>
+    <hyperlink r:id="rId81" location="12252" ref="E82"/>
     <hyperlink r:id="rId82" ref="E83"/>
     <hyperlink r:id="rId83" ref="E84"/>
     <hyperlink r:id="rId84" ref="E85"/>
     <hyperlink r:id="rId85" ref="E86"/>
     <hyperlink r:id="rId86" ref="E87"/>
     <hyperlink r:id="rId87" ref="E88"/>
-    <hyperlink r:id="rId88" ref="E89"/>
-    <hyperlink r:id="rId89" ref="E90"/>
+    <hyperlink r:id="rId88" location="Nfaq4.4.3.3" ref="E89"/>
+    <hyperlink r:id="rId89" location="Nfaq4.4.3.3" ref="E90"/>
     <hyperlink r:id="rId90" ref="E91"/>
     <hyperlink r:id="rId91" ref="E92"/>
     <hyperlink r:id="rId92" ref="E93"/>
@@ -12352,10 +12625,30 @@
     <hyperlink r:id="rId109" ref="E110"/>
     <hyperlink r:id="rId110" ref="E111"/>
     <hyperlink r:id="rId111" ref="E112"/>
+    <hyperlink r:id="rId112" ref="E113"/>
+    <hyperlink r:id="rId113" ref="E114"/>
+    <hyperlink r:id="rId114" ref="E115"/>
+    <hyperlink r:id="rId115" ref="E116"/>
+    <hyperlink r:id="rId116" ref="E117"/>
+    <hyperlink r:id="rId117" ref="E118"/>
+    <hyperlink r:id="rId118" ref="E119"/>
+    <hyperlink r:id="rId119" ref="E120"/>
+    <hyperlink r:id="rId120" ref="E121"/>
+    <hyperlink r:id="rId121" ref="E122"/>
+    <hyperlink r:id="rId122" ref="E123"/>
+    <hyperlink r:id="rId123" ref="E124"/>
+    <hyperlink r:id="rId124" ref="E125"/>
+    <hyperlink r:id="rId125" ref="E126"/>
+    <hyperlink r:id="rId126" ref="E127"/>
+    <hyperlink r:id="rId127" ref="E128"/>
+    <hyperlink r:id="rId128" ref="E129"/>
+    <hyperlink r:id="rId129" ref="E130"/>
+    <hyperlink r:id="rId130" ref="E131"/>
+    <hyperlink r:id="rId131" ref="E132"/>
   </hyperlinks>
-  <drawing r:id="rId112"/>
+  <drawing r:id="rId132"/>
   <tableParts count="1">
-    <tablePart r:id="rId114"/>
+    <tablePart r:id="rId134"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added more area units to AmericanUnits
</commit_message>
<xml_diff>
--- a/assets/code-files/american-units/UnitsSources.xlsx
+++ b/assets/code-files/american-units/UnitsSources.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="275">
   <si>
     <t>Unit Name</t>
   </si>
@@ -26,6 +26,54 @@
   </si>
   <si>
     <t>Source</t>
+  </si>
+  <si>
+    <t>Cost of a Costco Hot Dog</t>
+  </si>
+  <si>
+    <t>dollars</t>
+  </si>
+  <si>
+    <t>https://www.rd.com/article/reason-costco-hot-dogs-cheap/</t>
+  </si>
+  <si>
+    <t>Cost to see MLB baseball game</t>
+  </si>
+  <si>
+    <t>https://www.nytimes.com/athletic/2830372/2021/09/16/what-it-costs-for-every-mlb-teams-fans-to-attend-a-game-and-why-the-average-price-went-up-in-2021/</t>
+  </si>
+  <si>
+    <t>Average American Healthcare Spending in a Year</t>
+  </si>
+  <si>
+    <t>https://www.cms.gov/data-research/statistics-trends-and-reports/national-health-expenditure-data/historical</t>
+  </si>
+  <si>
+    <t>One second of U.S. Military</t>
+  </si>
+  <si>
+    <t>https://www.macrotrends.net/global-metrics/countries/usa/united-states/military-spending-defense-budget</t>
+  </si>
+  <si>
+    <t>Average college tuition in the U.S.</t>
+  </si>
+  <si>
+    <t>https://educationdata.org/average-cost-of-college</t>
+  </si>
+  <si>
+    <t>One minute of U.S. Military</t>
+  </si>
+  <si>
+    <t>One hour of U.S. Military</t>
+  </si>
+  <si>
+    <t>One day of U.S. Military</t>
+  </si>
+  <si>
+    <t>One month of U.S. Military</t>
+  </si>
+  <si>
+    <t>One year of U.S. Military</t>
   </si>
   <si>
     <t>Approximate Mass of a Bald Eagle's Feather</t>
@@ -487,16 +535,46 @@
     <t>Apple A4 Processer size</t>
   </si>
   <si>
+    <t>American Football Field Area</t>
+  </si>
+  <si>
+    <t>https://turftank.com/us/academy/how-big-is-a-football-field/</t>
+  </si>
+  <si>
+    <t>Floor Area of Boeing Everett Factory</t>
+  </si>
+  <si>
+    <t>https://science.howstuffworks.com/transport/flight/modern/boeings-everett-facility-is-largest-building-on-earth.htm</t>
+  </si>
+  <si>
+    <t>Washington D.C. Area</t>
+  </si>
+  <si>
+    <t>https://www.ebsco.com/research-starters/geography-and-cartography/washington-dc</t>
+  </si>
+  <si>
     <t>Rhode Island Area</t>
   </si>
   <si>
     <t>https://www.ri.gov/facts/history.php</t>
   </si>
   <si>
+    <t>Massachusetts Area</t>
+  </si>
+  <si>
+    <t>https://nchstats.com/map-of-massachusetts/</t>
+  </si>
+  <si>
     <t>Texas Area</t>
   </si>
   <si>
     <t>https://www.thestoryoftexas.com/resources/texas-facts/</t>
+  </si>
+  <si>
+    <t>Alaska Area</t>
+  </si>
+  <si>
+    <t>https://alaska.gov/Kids/learn/aboutgeography.htm</t>
   </si>
   <si>
     <t>United States Area</t>
@@ -873,54 +951,6 @@
   </si>
   <si>
     <t>https://www.lle.rochester.edu/omega-laser-facility/omega-ep/</t>
-  </si>
-  <si>
-    <t>One year of U.S. Military</t>
-  </si>
-  <si>
-    <t>dollars</t>
-  </si>
-  <si>
-    <t>https://www.macrotrends.net/global-metrics/countries/usa/united-states/military-spending-defense-budget</t>
-  </si>
-  <si>
-    <t>One month of U.S. Military</t>
-  </si>
-  <si>
-    <t>One day of U.S. Military</t>
-  </si>
-  <si>
-    <t>One hour of U.S. Military</t>
-  </si>
-  <si>
-    <t>One minute of U.S. Military</t>
-  </si>
-  <si>
-    <t>One second of U.S. Military</t>
-  </si>
-  <si>
-    <t>Average American Healthcare Spending in a Year</t>
-  </si>
-  <si>
-    <t>https://www.cms.gov/data-research/statistics-trends-and-reports/national-health-expenditure-data/historical</t>
-  </si>
-  <si>
-    <t>Average college tuition in the U.S.</t>
-  </si>
-  <si>
-    <t>https://educationdata.org/average-cost-of-college</t>
-  </si>
-  <si>
-    <t>Cost to see MLB baseball game</t>
-  </si>
-  <si>
-    <t>https://www.nytimes.com/athletic/2830372/2021/09/16/what-it-costs-for-every-mlb-teams-fans-to-attend-a-game-and-why-the-average-price-went-up-in-2021/</t>
-  </si>
-  <si>
-    <t>Cost of a Costco Hot Dog</t>
-  </si>
-  <si>
-    <t>https://www.rd.com/article/reason-costco-hot-dogs-cheap/</t>
   </si>
 </sst>
 </file>
@@ -979,7 +1009,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -994,7 +1024,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1300,7 +1330,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="55.38"/>
     <col customWidth="1" min="2" max="2" width="30.0"/>
-    <col customWidth="1" min="3" max="3" width="27.38"/>
+    <col customWidth="1" min="3" max="3" width="30.63"/>
     <col customWidth="1" min="4" max="4" width="35.25"/>
     <col customWidth="1" min="5" max="5" width="91.13"/>
   </cols>
@@ -1330,11 +1360,11 @@
         <v>6</v>
       </c>
       <c r="C2" s="3">
-        <v>0.06299888888</v>
+        <v>1.5</v>
       </c>
       <c r="D2" s="4">
         <f t="shared" ref="D2:D1014" si="1">IF(NOT(C2=0),1/C2,"")</f>
-        <v>15.87329583</v>
+        <v>0.6666666667</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>7</v>
@@ -1348,11 +1378,11 @@
         <v>6</v>
       </c>
       <c r="C3" s="3">
-        <v>0.175</v>
+        <v>63.25</v>
       </c>
       <c r="D3" s="4">
         <f t="shared" si="1"/>
-        <v>5.714285714</v>
+        <v>0.01581027668</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>9</v>
@@ -1366,11 +1396,11 @@
         <v>6</v>
       </c>
       <c r="C4" s="3">
-        <v>1.848</v>
+        <v>15474.0</v>
       </c>
       <c r="D4" s="4">
         <f t="shared" si="1"/>
-        <v>0.5411255411</v>
+        <v>0.00006462453147</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>11</v>
@@ -1384,11 +1414,11 @@
         <v>6</v>
       </c>
       <c r="C5" s="3">
-        <v>33.0</v>
+        <v>31624.4926433</v>
       </c>
       <c r="D5" s="4">
         <f t="shared" si="1"/>
-        <v>0.0303030303</v>
+        <v>0.00003162106065</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>13</v>
@@ -1402,11 +1432,11 @@
         <v>6</v>
       </c>
       <c r="C6" s="3">
-        <v>145.25</v>
+        <v>38270.0</v>
       </c>
       <c r="D6" s="4">
         <f t="shared" si="1"/>
-        <v>0.006884681583</v>
+        <v>0.00002613012804</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>15</v>
@@ -1420,429 +1450,429 @@
         <v>6</v>
       </c>
       <c r="C7" s="3">
-        <v>4309.13</v>
+        <v>1897469.5586</v>
       </c>
       <c r="D7" s="4">
         <f t="shared" si="1"/>
-        <v>0.0002320654053</v>
+        <v>0.0000005270176776</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="3">
-        <v>43200.0</v>
+        <v>1.13848173516E8</v>
       </c>
       <c r="D8" s="4">
         <f t="shared" si="1"/>
-        <v>0.00002314814815</v>
+        <v>0.000000008783627959</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="3">
-        <v>3020925.0</v>
+        <v>2.73235616438E9</v>
       </c>
       <c r="D9" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000003310244379</v>
+        <v>0.0000000003659844983</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="3">
-        <v>5.5E7</v>
+        <v>8.31091666667E10</v>
       </c>
       <c r="D10" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000001818181818</v>
+        <v>0</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="3">
-        <v>1.87E8</v>
+        <v>9.9731E11</v>
       </c>
       <c r="D11" s="4">
         <f t="shared" si="1"/>
-        <v>0.000000005347593583</v>
+        <v>0</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C12" s="3">
-        <v>3.0385E9</v>
+        <v>0.06299888888</v>
       </c>
       <c r="D12" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000000003291097581</v>
+        <v>15.87329583</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C13" s="3">
-        <v>1.062785E11</v>
+        <v>0.175</v>
       </c>
       <c r="D13" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5.714285714</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C14" s="3">
-        <v>3.6E11</v>
+        <v>1.848</v>
       </c>
       <c r="D14" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.5411255411</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C15" s="3">
-        <v>6.6405922968E12</v>
+        <v>33.0</v>
       </c>
       <c r="D15" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>33</v>
+        <v>0.0303030303</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="3">
+        <v>145.25</v>
+      </c>
+      <c r="D16" s="4">
+        <f t="shared" si="1"/>
+        <v>0.006884681583</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="3">
+        <v>4309.13</v>
+      </c>
+      <c r="D17" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0002320654053</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="3">
+      <c r="B18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="3">
+        <v>43200.0</v>
+      </c>
+      <c r="D18" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00002314814815</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="3">
+        <v>3020925.0</v>
+      </c>
+      <c r="D19" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000003310244379</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="3">
+        <v>5.5E7</v>
+      </c>
+      <c r="D20" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00000001818181818</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="3">
+        <v>1.87E8</v>
+      </c>
+      <c r="D21" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000005347593583</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="3">
+        <v>3.0385E9</v>
+      </c>
+      <c r="D22" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000000003291097581</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="3">
+        <v>1.062785E11</v>
+      </c>
+      <c r="D23" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="3">
+        <v>3.6E11</v>
+      </c>
+      <c r="D24" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="3">
+        <v>6.6405922968E12</v>
+      </c>
+      <c r="D25" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C26" s="3">
         <f>7.64*10^14</f>
         <v>764000000000000</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D26" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E16" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="3">
+      <c r="E26" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" s="3">
         <v>3.44468E-11</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D27" s="4">
         <f t="shared" si="1"/>
         <v>29030272768</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="3">
-        <v>162.461421789</v>
-      </c>
-      <c r="D18" s="4">
-        <f t="shared" si="1"/>
-        <v>0.006155307451</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="3">
-        <v>475.892</v>
-      </c>
-      <c r="D19" s="4">
-        <f t="shared" si="1"/>
-        <v>0.002101317106</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" s="3">
-        <v>5548.007</v>
-      </c>
-      <c r="D20" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000180244906</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="3">
-        <v>54392.0</v>
-      </c>
-      <c r="D21" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00001838505663</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C22" s="3">
-        <v>502080.0</v>
-      </c>
-      <c r="D22" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000001991714468</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C23" s="3">
-        <v>2845000.0</v>
-      </c>
-      <c r="D23" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000003514938489</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C24" s="3">
-        <v>3.3E7</v>
-      </c>
-      <c r="D24" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000000303030303</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" s="3">
-        <v>1.32E8</v>
-      </c>
-      <c r="D25" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000000007575757576</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="1" t="s">
+      <c r="E27" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" s="3">
-        <v>2.092E9</v>
-      </c>
-      <c r="D26" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000000004780114723</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="27" ht="22.5" customHeight="1">
-      <c r="A27" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" s="3">
-        <v>4.6024E10</v>
-      </c>
-      <c r="D27" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="3">
+        <v>162.461421789</v>
+      </c>
+      <c r="D28" s="4">
+        <f t="shared" si="1"/>
+        <v>0.006155307451</v>
+      </c>
+      <c r="E28" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C28" s="3">
-        <v>6.276E13</v>
-      </c>
-      <c r="D28" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="3">
+        <v>475.892</v>
+      </c>
+      <c r="D29" s="4">
+        <f t="shared" si="1"/>
+        <v>0.002101317106</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" s="3">
-        <v>4.35136E16</v>
-      </c>
-      <c r="D29" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="3">
+        <v>5548.007</v>
+      </c>
+      <c r="D30" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000180244906</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" s="3">
-        <v>1.00416E17</v>
-      </c>
-      <c r="D30" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
@@ -1850,14 +1880,14 @@
         <v>61</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C31" s="3">
-        <v>7.07945784384137E17</v>
+        <v>54392.0</v>
       </c>
       <c r="D31" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.00001838505663</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>62</v>
@@ -1868,1751 +1898,1750 @@
         <v>63</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C32" s="3">
-        <v>4.3321136E18</v>
+        <v>502080.0</v>
       </c>
       <c r="D32" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>64</v>
+        <v>0.000001991714468</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="33" ht="22.5" customHeight="1">
       <c r="A33" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="3">
+        <v>2845000.0</v>
+      </c>
+      <c r="D33" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000003514938489</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C33" s="3">
-        <v>0.04063992</v>
-      </c>
-      <c r="D33" s="4">
-        <f t="shared" si="1"/>
-        <v>24.60634765</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C34" s="3">
-        <v>0.221801</v>
+        <v>3.3E7</v>
       </c>
       <c r="D34" s="4">
         <f t="shared" si="1"/>
-        <v>4.508545949</v>
+        <v>0.0000000303030303</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" ht="22.5" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C35" s="3">
-        <v>4.5</v>
+        <v>1.32E8</v>
       </c>
       <c r="D35" s="4">
         <f t="shared" si="1"/>
-        <v>0.2222222222</v>
+        <v>0.000000007575757576</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" ht="22.5" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C36" s="3">
-        <v>5.0275</v>
+        <v>2.092E9</v>
       </c>
       <c r="D36" s="4">
         <f t="shared" si="1"/>
-        <v>0.1989060169</v>
+        <v>0.0000000004780114723</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" ht="22.5" customHeight="1">
-      <c r="A37" s="1" t="s">
-        <v>74</v>
+      <c r="A37" s="7" t="s">
+        <v>71</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C37" s="3">
-        <v>27.2353</v>
+        <v>4.6024E10</v>
       </c>
       <c r="D37" s="4">
         <f t="shared" si="1"/>
-        <v>0.0367170547</v>
+        <v>0</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" ht="22.5" customHeight="1">
       <c r="A38" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C38" s="3">
-        <v>1214.793</v>
+        <v>6.276E13</v>
       </c>
       <c r="D38" s="4">
         <f t="shared" si="1"/>
-        <v>0.0008231855139</v>
+        <v>0</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" ht="22.5" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C39" s="3">
-        <v>9344.56</v>
+        <v>4.35136E16</v>
       </c>
       <c r="D39" s="4">
         <f t="shared" si="1"/>
-        <v>0.0001070141344</v>
+        <v>0</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="40" ht="22.5" customHeight="1">
       <c r="A40" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C40" s="3">
-        <v>47968.74</v>
+        <v>1.00416E17</v>
       </c>
       <c r="D40" s="4">
         <f t="shared" si="1"/>
-        <v>0.00002084690988</v>
+        <v>0</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41" ht="22.5" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C41" s="3">
-        <v>187700.0</v>
+        <v>7.07945784384137E17</v>
       </c>
       <c r="D41" s="4">
         <f t="shared" si="1"/>
-        <v>0.000005327650506</v>
+        <v>0</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" ht="22.5" customHeight="1">
       <c r="A42" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C42" s="3">
-        <v>959941.1</v>
+        <v>4.3321136E18</v>
       </c>
       <c r="D42" s="4">
         <f t="shared" si="1"/>
-        <v>0.000001041730581</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>85</v>
+        <v>0</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="43" ht="22.5" customHeight="1">
       <c r="A43" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="C43" s="3">
-        <v>1.9093578E7</v>
+        <v>0.04063992</v>
       </c>
       <c r="D43" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000005237363055</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>87</v>
+        <v>24.60634765</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="44" ht="22.5" customHeight="1">
       <c r="A44" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="C44" s="3">
-        <v>3.66E9</v>
+        <v>0.221801</v>
       </c>
       <c r="D44" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000000002732240437</v>
+        <v>4.508545949</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" ht="22.5" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="C45" s="3">
-        <v>2.25247011911E10</v>
+        <v>4.5</v>
       </c>
       <c r="D45" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.2222222222</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46" ht="22.5" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="C46" s="3">
-        <v>4.81744222615434E13</v>
+        <v>5.0275</v>
       </c>
       <c r="D46" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.1989060169</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" ht="22.5" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="C47" s="3">
-        <v>1.31180417045093E14</v>
+        <v>27.2353</v>
       </c>
       <c r="D47" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.0367170547</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" ht="22.5" customHeight="1">
       <c r="A48" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="C48" s="3">
-        <v>1.678752E16</v>
+        <v>1214.793</v>
       </c>
       <c r="D48" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>97</v>
+        <v>0.0008231855139</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="49" ht="22.5" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C49" s="3">
-        <v>7.6E-4</v>
+        <v>9344.56</v>
       </c>
       <c r="D49" s="4">
         <f t="shared" si="1"/>
-        <v>1315.789474</v>
+        <v>0.0001070141344</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" ht="22.5" customHeight="1">
       <c r="A50" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C50" s="3">
-        <v>0.0085</v>
+        <v>47968.74</v>
       </c>
       <c r="D50" s="4">
         <f t="shared" si="1"/>
-        <v>117.6470588</v>
+        <v>0.00002084690988</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="51" ht="22.5" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B51" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C51" s="3">
+        <v>187700.0</v>
+      </c>
+      <c r="D51" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000005327650506</v>
+      </c>
+      <c r="E51" s="5" t="s">
         <v>99</v>
-      </c>
-      <c r="C51" s="3">
-        <v>0.0762</v>
-      </c>
-      <c r="D51" s="4">
-        <f t="shared" si="1"/>
-        <v>13.12335958</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="52" ht="22.5" customHeight="1">
       <c r="A52" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C52" s="3">
-        <v>0.83185</v>
+        <v>959941.1</v>
       </c>
       <c r="D52" s="4">
         <f t="shared" si="1"/>
-        <v>1.202139809</v>
+        <v>0.000001041730581</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="53" ht="22.5" customHeight="1">
       <c r="A53" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C53" s="3">
-        <v>1.87</v>
+        <v>1.9093578E7</v>
       </c>
       <c r="D53" s="4">
         <f t="shared" si="1"/>
-        <v>0.5347593583</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>108</v>
+        <v>0.00000005237363055</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="54" ht="22.5" customHeight="1">
       <c r="A54" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C54" s="3">
-        <v>2.0</v>
+        <v>3.66E9</v>
       </c>
       <c r="D54" s="4">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0.0000000002732240437</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="55" ht="22.5" customHeight="1">
       <c r="A55" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C55" s="3">
-        <v>5.31876</v>
+        <v>2.25247011911E10</v>
       </c>
       <c r="D55" s="4">
         <f t="shared" si="1"/>
-        <v>0.1880137476</v>
+        <v>0</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" ht="22.5" customHeight="1">
       <c r="A56" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C56" s="3">
-        <v>109.75</v>
+        <v>4.81744222615434E13</v>
       </c>
       <c r="D56" s="4">
         <f t="shared" si="1"/>
-        <v>0.009111617312</v>
+        <v>0</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="57" ht="22.5" customHeight="1">
       <c r="A57" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C57" s="3">
-        <v>380.0</v>
+        <v>1.31180417045093E14</v>
       </c>
       <c r="D57" s="4">
         <f t="shared" si="1"/>
-        <v>0.002631578947</v>
+        <v>0</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="58" ht="22.5" customHeight="1">
       <c r="A58" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C58" s="3">
-        <v>77248.5</v>
+        <v>1.678752E16</v>
       </c>
       <c r="D58" s="4">
         <f t="shared" si="1"/>
-        <v>0.00001294523518</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>118</v>
+        <v>0</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="59" ht="22.5" customHeight="1">
       <c r="A59" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C59" s="3">
-        <v>455444.0</v>
+        <v>7.6E-4</v>
       </c>
       <c r="D59" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000219565962</v>
+        <v>1315.789474</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="60" ht="22.5" customHeight="1">
       <c r="A60" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C60" s="3">
-        <v>4500000.0</v>
+        <v>0.0085</v>
       </c>
       <c r="D60" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000002222222222</v>
+        <v>117.6470588</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="61" ht="22.5" customHeight="1">
       <c r="A61" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C61" s="3">
-        <v>1.3E7</v>
+        <v>0.0762</v>
       </c>
       <c r="D61" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000007692307692</v>
+        <v>13.12335958</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="62" ht="22.5" customHeight="1">
       <c r="A62" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C62" s="3">
-        <v>1.51864E8</v>
+        <v>0.83185</v>
       </c>
       <c r="D62" s="4">
         <f t="shared" si="1"/>
-        <v>0.000000006584839067</v>
+        <v>1.202139809</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="63" ht="22.5" customHeight="1">
       <c r="A63" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C63" s="3">
-        <v>2.896678140998E10</v>
+        <v>1.87</v>
       </c>
       <c r="D63" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.5347593583</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="64" ht="22.5" customHeight="1">
       <c r="A64" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C64" s="3">
-        <v>5.1499008E12</v>
+        <v>2.0</v>
       </c>
       <c r="D64" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="65" ht="22.5" customHeight="1">
       <c r="A65" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="C65" s="3">
-        <v>7.11E-19</v>
+        <v>5.31876</v>
       </c>
       <c r="D65" s="4">
         <f t="shared" si="1"/>
-        <v>1.40647E+18</v>
+        <v>0.1880137476</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="66" ht="22.5" customHeight="1">
       <c r="A66" s="1" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="C66" s="3">
-        <v>7.2E-5</v>
+        <v>109.75</v>
       </c>
       <c r="D66" s="4">
         <f t="shared" si="1"/>
-        <v>13888.88889</v>
+        <v>0.009111617312</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>102</v>
+        <v>130</v>
       </c>
     </row>
     <row r="67" ht="22.5" customHeight="1">
       <c r="A67" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C67" s="3">
+        <v>380.0</v>
+      </c>
+      <c r="D67" s="4">
+        <f t="shared" si="1"/>
+        <v>0.002631578947</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="68" ht="22.5" customHeight="1">
+      <c r="A68" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C68" s="3">
+        <v>77248.5</v>
+      </c>
+      <c r="D68" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00001294523518</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69" ht="22.5" customHeight="1">
+      <c r="A69" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B67" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C67" s="3">
+      <c r="B69" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C69" s="3">
+        <v>455444.0</v>
+      </c>
+      <c r="D69" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00000219565962</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="70" ht="22.5" customHeight="1">
+      <c r="A70" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C70" s="3">
+        <v>4500000.0</v>
+      </c>
+      <c r="D70" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000002222222222</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="71" ht="22.5" customHeight="1">
+      <c r="A71" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C71" s="3">
+        <v>1.3E7</v>
+      </c>
+      <c r="D71" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00000007692307692</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="72" ht="22.5" customHeight="1">
+      <c r="A72" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C72" s="3">
+        <v>1.51864E8</v>
+      </c>
+      <c r="D72" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000006584839067</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="73" ht="22.5" customHeight="1">
+      <c r="A73" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C73" s="3">
+        <v>2.896678140998E10</v>
+      </c>
+      <c r="D73" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="74" ht="22.5" customHeight="1">
+      <c r="A74" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C74" s="3">
+        <v>5.1499008E12</v>
+      </c>
+      <c r="D74" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="75" ht="22.5" customHeight="1">
+      <c r="A75" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C75" s="3">
+        <v>7.11E-19</v>
+      </c>
+      <c r="D75" s="4">
+        <f t="shared" si="1"/>
+        <v>1.40647E+18</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="76" ht="22.5" customHeight="1">
+      <c r="A76" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C76" s="3">
+        <v>7.2E-5</v>
+      </c>
+      <c r="D76" s="4">
+        <f t="shared" si="1"/>
+        <v>13888.88889</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="77" ht="22.5" customHeight="1">
+      <c r="A77" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C77" s="3">
+        <v>5351.2151</v>
+      </c>
+      <c r="D77" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0001868734449</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="78" ht="22.5" customHeight="1">
+      <c r="A78" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C78" s="3">
+        <v>397806.0</v>
+      </c>
+      <c r="D78" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000002513788128</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="79" ht="22.5" customHeight="1">
+      <c r="A79" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C79" s="3">
+        <v>1.761E8</v>
+      </c>
+      <c r="D79" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000005678591709</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="80" ht="22.5" customHeight="1">
+      <c r="A80" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C80" s="3">
         <f>2.70654*10^9</f>
         <v>2706540000</v>
       </c>
-      <c r="D67" s="4">
+      <c r="D80" s="4">
         <f t="shared" si="1"/>
         <v>0.0000000003694754188</v>
       </c>
-      <c r="E67" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="68" ht="22.5" customHeight="1">
-      <c r="A68" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C68" s="8">
+      <c r="E80" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="81" ht="22.5" customHeight="1">
+      <c r="A81" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C81" s="3">
+        <v>2.733732E10</v>
+      </c>
+      <c r="D81" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E81" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="82" ht="22.5" customHeight="1">
+      <c r="A82" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C82" s="8">
         <f>6.9566045*10^11</f>
         <v>695660450000</v>
       </c>
-      <c r="D68" s="4">
+      <c r="D82" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E68" s="5" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="69" ht="22.5" customHeight="1">
-      <c r="A69" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C69" s="3">
-        <v>9.866624456E12</v>
-      </c>
-      <c r="D69" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E69" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="70" ht="22.5" customHeight="1">
-      <c r="A70" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C70" s="3">
-        <v>0.002</v>
-      </c>
-      <c r="D70" s="4">
-        <f t="shared" si="1"/>
-        <v>500</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="71" ht="22.5" customHeight="1">
-      <c r="A71" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C71" s="3">
-        <v>0.02</v>
-      </c>
-      <c r="D71" s="4">
-        <f t="shared" si="1"/>
-        <v>50</v>
-      </c>
-      <c r="E71" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="72" ht="22.5" customHeight="1">
-      <c r="A72" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C72" s="3">
-        <v>0.10289818517</v>
-      </c>
-      <c r="D72" s="4">
-        <f t="shared" si="1"/>
-        <v>9.718344384</v>
-      </c>
-      <c r="E72" s="6" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="73" ht="22.5" customHeight="1">
-      <c r="A73" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C73" s="3">
-        <v>0.735</v>
-      </c>
-      <c r="D73" s="4">
-        <f t="shared" si="1"/>
-        <v>1.360544218</v>
-      </c>
-      <c r="E73" s="6" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="74" ht="22.5" customHeight="1">
-      <c r="A74" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C74" s="3">
-        <v>956.368</v>
-      </c>
-      <c r="D74" s="4">
-        <f t="shared" si="1"/>
-        <v>0.001045622606</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="75" ht="22.5" customHeight="1">
-      <c r="A75" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C75" s="3">
-        <v>7117.155</v>
-      </c>
-      <c r="D75" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0001405055812</v>
-      </c>
-      <c r="E75" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="76" ht="22.5" customHeight="1">
-      <c r="A76" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C76" s="3">
-        <v>13172.0</v>
-      </c>
-      <c r="D76" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00007591861524</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="77" ht="22.5" customHeight="1">
-      <c r="A77" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C77" s="3">
-        <v>40000.0</v>
-      </c>
-      <c r="D77" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000025</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="78" ht="22.5" customHeight="1">
-      <c r="A78" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C78" s="3">
-        <v>511545.484</v>
-      </c>
-      <c r="D78" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000001954860381</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="79" ht="22.5" customHeight="1">
-      <c r="A79" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C79" s="3">
-        <v>1668083.1</v>
-      </c>
-      <c r="D79" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000000599490517</v>
-      </c>
-      <c r="E79" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="80" ht="22.5" customHeight="1">
-      <c r="A80" s="1" t="s">
+      <c r="E82" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C80" s="3">
-        <v>3.45E7</v>
-      </c>
-      <c r="D80" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00000002898550725</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="81" ht="22.5" customHeight="1">
-      <c r="A81" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C81" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="D81" s="4">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="E81" s="5" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="82" ht="22.5" customHeight="1">
-      <c r="A82" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C82" s="3">
-        <v>86.0</v>
-      </c>
-      <c r="D82" s="4">
-        <f t="shared" si="1"/>
-        <v>0.01162790698</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="83" ht="22.5" customHeight="1">
       <c r="A83" s="1" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="C83" s="3">
-        <v>120.0</v>
+        <v>1.5188001E12</v>
       </c>
       <c r="D83" s="4">
         <f t="shared" si="1"/>
-        <v>0.008333333333</v>
+        <v>0</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="84" ht="22.5" customHeight="1">
       <c r="A84" s="1" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="C84" s="3">
-        <v>258553.4</v>
+        <v>9.866624456E12</v>
       </c>
       <c r="D84" s="4">
         <f t="shared" si="1"/>
-        <v>0.000003867672984</v>
+        <v>0</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
     </row>
     <row r="85" ht="22.5" customHeight="1">
       <c r="A85" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C85" s="3">
-        <v>2384190.0</v>
+        <v>0.002</v>
       </c>
       <c r="D85" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000004194296595</v>
+        <v>500</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="86" ht="22.5" customHeight="1">
       <c r="A86" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C86" s="3">
-        <v>2.8E7</v>
+        <v>0.02</v>
       </c>
       <c r="D86" s="4">
         <f t="shared" si="1"/>
-        <v>0.00000003571428571</v>
+        <v>50</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="87" ht="22.5" customHeight="1">
       <c r="A87" s="1" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C87" s="3">
-        <v>4.82633E8</v>
+        <v>0.10289818517</v>
       </c>
       <c r="D87" s="4">
         <f t="shared" si="1"/>
-        <v>0.000000002071967727</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>178</v>
+        <v>9.718344384</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="88" ht="22.5" customHeight="1">
       <c r="A88" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C88" s="3">
-        <v>5.0E12</v>
+        <v>0.735</v>
       </c>
       <c r="D88" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>180</v>
+        <v>1.360544218</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="89" ht="22.5" customHeight="1">
       <c r="A89" s="1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C89" s="3">
-        <v>5.4E14</v>
+        <v>956.368</v>
       </c>
       <c r="D89" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.001045622606</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="90" ht="22.5" customHeight="1">
       <c r="A90" s="1" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C90" s="3">
-        <v>6.5E15</v>
+        <v>7117.155</v>
       </c>
       <c r="D90" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.0001405055812</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="91" ht="22.5" customHeight="1">
       <c r="A91" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="3">
+        <v>13172.0</v>
+      </c>
+      <c r="D91" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00007591861524</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="92" ht="22.5" customHeight="1">
+      <c r="A92" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C92" s="3">
+        <v>40000.0</v>
+      </c>
+      <c r="D92" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000025</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="93" ht="22.5" customHeight="1">
+      <c r="A93" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B93" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C93" s="3">
+        <v>511545.484</v>
+      </c>
+      <c r="D93" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000001954860381</v>
+      </c>
+      <c r="E93" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="C91" s="8">
+    </row>
+    <row r="94" ht="22.5" customHeight="1">
+      <c r="A94" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C94" s="3">
+        <v>1668083.1</v>
+      </c>
+      <c r="D94" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000599490517</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="95" ht="22.5" customHeight="1">
+      <c r="A95" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C95" s="3">
+        <v>3.45E7</v>
+      </c>
+      <c r="D95" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00000002898550725</v>
+      </c>
+      <c r="E95" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="96" ht="22.5" customHeight="1">
+      <c r="A96" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C96" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D96" s="4">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E96" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="97" ht="22.5" customHeight="1">
+      <c r="A97" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C97" s="3">
+        <v>86.0</v>
+      </c>
+      <c r="D97" s="4">
+        <f t="shared" si="1"/>
+        <v>0.01162790698</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="98" ht="22.5" customHeight="1">
+      <c r="A98" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C98" s="3">
+        <v>120.0</v>
+      </c>
+      <c r="D98" s="4">
+        <f t="shared" si="1"/>
+        <v>0.008333333333</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="99" ht="22.5" customHeight="1">
+      <c r="A99" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C99" s="3">
+        <v>258553.4</v>
+      </c>
+      <c r="D99" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000003867672984</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="100" ht="22.5" customHeight="1">
+      <c r="A100" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C100" s="3">
+        <v>2384190.0</v>
+      </c>
+      <c r="D100" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000004194296595</v>
+      </c>
+      <c r="E100" s="5" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="101" ht="22.5" customHeight="1">
+      <c r="A101" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C101" s="3">
+        <v>2.8E7</v>
+      </c>
+      <c r="D101" s="4">
+        <f t="shared" si="1"/>
+        <v>0.00000003571428571</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="102" ht="22.5" customHeight="1">
+      <c r="A102" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C102" s="3">
+        <v>4.82633E8</v>
+      </c>
+      <c r="D102" s="4">
+        <f t="shared" si="1"/>
+        <v>0.000000002071967727</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="103" ht="22.5" customHeight="1">
+      <c r="A103" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C103" s="3">
+        <v>5.0E12</v>
+      </c>
+      <c r="D103" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E103" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="104" ht="22.5" customHeight="1">
+      <c r="A104" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C104" s="3">
+        <v>5.4E14</v>
+      </c>
+      <c r="D104" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E104" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="105" ht="22.5" customHeight="1">
+      <c r="A105" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C105" s="3">
+        <v>6.5E15</v>
+      </c>
+      <c r="D105" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E105" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="106" ht="22.5" customHeight="1">
+      <c r="A106" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C106" s="8">
         <f>10^-8</f>
         <v>0.00000001</v>
       </c>
-      <c r="D91" s="4">
+      <c r="D106" s="4">
         <f t="shared" si="1"/>
         <v>100000000</v>
       </c>
-      <c r="E91" s="5" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="92" ht="22.5" customHeight="1">
-      <c r="A92" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C92" s="3">
+      <c r="E106" s="5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="107" ht="22.5" customHeight="1">
+      <c r="A107" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C107" s="3">
         <f>1/100</f>
         <v>0.01</v>
       </c>
-      <c r="D92" s="4">
+      <c r="D107" s="4">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="E92" s="5" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="93" ht="22.5" customHeight="1">
-      <c r="A93" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C93" s="8">
+      <c r="E107" s="5" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="108" ht="22.5" customHeight="1">
+      <c r="A108" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C108" s="8">
         <f>1/3</f>
         <v>0.3333333333</v>
       </c>
-      <c r="D93" s="4">
+      <c r="D108" s="4">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="E93" s="5" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="94" ht="22.5" customHeight="1">
-      <c r="A94" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C94" s="3">
-        <v>10.0</v>
-      </c>
-      <c r="D94" s="4">
-        <f t="shared" si="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="E94" s="9" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="95" ht="22.5" customHeight="1">
-      <c r="A95" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C95" s="3">
-        <v>103.0</v>
-      </c>
-      <c r="D95" s="4">
-        <f t="shared" si="1"/>
-        <v>0.009708737864</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="96" ht="22.5" customHeight="1">
-      <c r="A96" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B96" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C96" s="3">
-        <v>1200.0</v>
-      </c>
-      <c r="D96" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0008333333333</v>
-      </c>
-      <c r="E96" s="5" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="97" ht="22.5" customHeight="1">
-      <c r="A97" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C97" s="3">
-        <v>12600.0</v>
-      </c>
-      <c r="D97" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00007936507937</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="98" ht="22.5" customHeight="1">
-      <c r="A98" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="B98" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C98" s="3">
-        <v>154440.0</v>
-      </c>
-      <c r="D98" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000006475006475</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="99" ht="22.5" customHeight="1">
-      <c r="A99" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C99" s="3">
-        <v>2637000.0</v>
-      </c>
-      <c r="D99" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000003792188093</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="100" ht="22.5" customHeight="1">
-      <c r="A100" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C100" s="3">
-        <v>1.823E7</v>
-      </c>
-      <c r="D100" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00000005485463522</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="101" ht="22.5" customHeight="1">
-      <c r="A101" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C101" s="3">
-        <v>6.312E7</v>
-      </c>
-      <c r="D101" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00000001584283904</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="102" ht="22.5" customHeight="1">
-      <c r="A102" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C102" s="3">
-        <v>1.893E8</v>
-      </c>
-      <c r="D102" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00000000528262018</v>
-      </c>
-      <c r="E102" s="5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="103" ht="22.5" customHeight="1">
-      <c r="A103" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C103" s="3">
-        <v>2.0123E8</v>
-      </c>
-      <c r="D103" s="4">
-        <f t="shared" si="1"/>
-        <v>0.000000004969437957</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="104" ht="22.5" customHeight="1">
-      <c r="A104" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C104" s="3">
-        <v>7.88728E9</v>
-      </c>
-      <c r="D104" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000000001267864207</v>
-      </c>
-      <c r="E104" s="5" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="105" ht="22.5" customHeight="1">
-      <c r="A105" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C105" s="3">
-        <v>1.684092E10</v>
-      </c>
-      <c r="D105" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E105" s="5" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="106" ht="22.5" customHeight="1">
-      <c r="A106" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C106" s="3">
-        <v>9.4608E11</v>
-      </c>
-      <c r="D106" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E106" s="5" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="107" ht="22.5" customHeight="1">
-      <c r="A107" s="1" t="s">
+      <c r="E108" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="C107" s="3">
-        <v>1.0233782E15</v>
-      </c>
-      <c r="D107" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E107" s="9" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="108" ht="22.5" customHeight="1">
-      <c r="A108" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="B108" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="C108" s="3">
-        <v>50.0</v>
-      </c>
-      <c r="D108" s="4">
-        <f t="shared" si="1"/>
-        <v>0.02</v>
-      </c>
-      <c r="E108" s="5" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="109" ht="22.5" customHeight="1">
       <c r="A109" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C109" s="3">
-        <v>60.0</v>
+        <v>10.0</v>
       </c>
       <c r="D109" s="4">
         <f t="shared" si="1"/>
-        <v>0.01666666667</v>
-      </c>
-      <c r="E109" s="5" t="s">
-        <v>222</v>
+        <v>0.1</v>
+      </c>
+      <c r="E109" s="9" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="110" ht="22.5" customHeight="1">
       <c r="A110" s="1" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C110" s="3">
-        <v>9334.11285138</v>
+        <v>103.0</v>
       </c>
       <c r="D110" s="4">
         <f t="shared" si="1"/>
-        <v>0.0001071339093</v>
+        <v>0.009708737864</v>
       </c>
       <c r="E110" s="5" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="111" ht="22.5" customHeight="1">
-      <c r="A111" s="7" t="s">
-        <v>225</v>
+      <c r="A111" s="1" t="s">
+        <v>221</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C111" s="3">
-        <v>100000.0</v>
+        <v>1200.0</v>
       </c>
       <c r="D111" s="4">
         <f t="shared" si="1"/>
-        <v>0.00001</v>
+        <v>0.0008333333333</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="112" ht="22.5" customHeight="1">
       <c r="A112" s="1" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C112" s="3">
-        <v>514849.0</v>
+        <v>12600.0</v>
       </c>
       <c r="D112" s="4">
         <f t="shared" si="1"/>
-        <v>0.000001942317068</v>
+        <v>0.00007936507937</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="113" ht="22.5" customHeight="1">
       <c r="A113" s="1" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C113" s="3">
-        <v>1265058.0</v>
+        <v>154440.0</v>
       </c>
       <c r="D113" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000007904775908</v>
+        <v>0.000006475006475</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="114" ht="22.5" customHeight="1">
       <c r="A114" s="1" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C114" s="3">
-        <v>2.5742456E7</v>
+        <v>2637000.0</v>
       </c>
       <c r="D114" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000000388463323</v>
+        <v>0.0000003792188093</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="115" ht="22.5" customHeight="1">
       <c r="A115" s="1" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C115" s="3">
-        <v>1.91229675E8</v>
+        <v>1.823E7</v>
       </c>
       <c r="D115" s="4">
         <f t="shared" si="1"/>
-        <v>0.000000005229313913</v>
+        <v>0.00000005485463522</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="116" ht="22.5" customHeight="1">
       <c r="A116" s="1" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C116" s="3">
-        <v>2.08E9</v>
+        <v>6.312E7</v>
       </c>
       <c r="D116" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000000004807692308</v>
+        <v>0.00000001584283904</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="117" ht="22.5" customHeight="1">
       <c r="A117" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C117" s="3">
-        <v>1.2E10</v>
+        <v>1.893E8</v>
       </c>
       <c r="D117" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.00000000528262018</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="118" ht="22.5" customHeight="1">
       <c r="A118" s="1" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C118" s="3">
-        <v>8.81529680365E10</v>
+        <v>2.0123E8</v>
       </c>
       <c r="D118" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.000000004969437957</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
     </row>
     <row r="119" ht="22.5" customHeight="1">
       <c r="A119" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C119" s="3">
-        <v>2.39E11</v>
+        <v>7.88728E9</v>
       </c>
       <c r="D119" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E119" s="9" t="s">
-        <v>242</v>
+        <v>0.0000000001267864207</v>
+      </c>
+      <c r="E119" s="5" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="120" ht="22.5" customHeight="1">
       <c r="A120" s="1" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C120" s="3">
-        <v>3.2552635E12</v>
+        <v>1.684092E10</v>
       </c>
       <c r="D120" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="121" ht="22.5" customHeight="1">
       <c r="A121" s="1" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="C121" s="8">
-        <f>3*10^14</f>
-        <v>300000000000000</v>
+        <v>211</v>
+      </c>
+      <c r="C121" s="3">
+        <v>9.4608E11</v>
       </c>
       <c r="D121" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="122" ht="22.5" customHeight="1">
       <c r="A122" s="1" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C122" s="3">
-        <v>1.4285714E15</v>
+        <v>1.0233782E15</v>
       </c>
       <c r="D122" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E122" s="5" t="s">
-        <v>248</v>
+      <c r="E122" s="9" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="123" ht="22.5" customHeight="1">
       <c r="A123" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C123" s="3">
-        <v>9.9731E11</v>
+        <v>50.0</v>
       </c>
       <c r="D123" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E123" s="5" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="124" ht="22.5" customHeight="1">
       <c r="A124" s="1" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C124" s="3">
-        <v>8.31091666667E10</v>
+        <v>60.0</v>
       </c>
       <c r="D124" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.01666666667</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="125" ht="22.5" customHeight="1">
       <c r="A125" s="1" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B125" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C125" s="3">
+        <v>9334.11285138</v>
+      </c>
+      <c r="D125" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0001071339093</v>
+      </c>
+      <c r="E125" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="C125" s="3">
-        <v>2.73235616438E9</v>
-      </c>
-      <c r="D125" s="4">
-        <f t="shared" si="1"/>
-        <v>0.0000000003659844983</v>
-      </c>
-      <c r="E125" s="5" t="s">
+    </row>
+    <row r="126" ht="22.5" customHeight="1">
+      <c r="A126" s="7" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="126" ht="22.5" customHeight="1">
-      <c r="A126" s="1" t="s">
-        <v>254</v>
-      </c>
       <c r="B126" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C126" s="3">
-        <v>1.13848173516E8</v>
+        <v>100000.0</v>
       </c>
       <c r="D126" s="4">
         <f t="shared" si="1"/>
-        <v>0.000000008783627959</v>
+        <v>0.00001</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="127" ht="22.5" customHeight="1">
       <c r="A127" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C127" s="3">
-        <v>1897469.5586</v>
+        <v>514849.0</v>
       </c>
       <c r="D127" s="4">
         <f t="shared" si="1"/>
-        <v>0.0000005270176776</v>
+        <v>0.000001942317068</v>
       </c>
       <c r="E127" s="5" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="128" ht="22.5" customHeight="1">
       <c r="A128" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C128" s="3">
+        <v>1265058.0</v>
+      </c>
+      <c r="D128" s="4">
+        <f t="shared" si="1"/>
+        <v>0.0000007904775908</v>
+      </c>
+      <c r="E128" s="5" t="s">
         <v>256</v>
-      </c>
-      <c r="B128" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="C128" s="3">
-        <v>31624.4926433</v>
-      </c>
-      <c r="D128" s="4">
-        <f t="shared" si="1"/>
-        <v>0.00003162106065</v>
-      </c>
-      <c r="E128" s="5" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="129" ht="22.5" customHeight="1">
@@ -3620,14 +3649,14 @@
         <v>257</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C129" s="3">
-        <v>15474.0</v>
+        <v>2.5742456E7</v>
       </c>
       <c r="D129" s="4">
         <f t="shared" si="1"/>
-        <v>0.00006462453147</v>
+        <v>0.0000000388463323</v>
       </c>
       <c r="E129" s="5" t="s">
         <v>258</v>
@@ -3638,14 +3667,14 @@
         <v>259</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C130" s="3">
-        <v>38270.0</v>
+        <v>1.91229675E8</v>
       </c>
       <c r="D130" s="4">
         <f t="shared" si="1"/>
-        <v>0.00002613012804</v>
+        <v>0.000000005229313913</v>
       </c>
       <c r="E130" s="5" t="s">
         <v>260</v>
@@ -3656,14 +3685,14 @@
         <v>261</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C131" s="3">
-        <v>63.25</v>
+        <v>2.08E9</v>
       </c>
       <c r="D131" s="4">
         <f t="shared" si="1"/>
-        <v>0.01581027668</v>
+        <v>0.0000000004807692308</v>
       </c>
       <c r="E131" s="5" t="s">
         <v>262</v>
@@ -3674,68 +3703,109 @@
         <v>263</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C132" s="3">
-        <v>1.5</v>
+        <v>1.2E10</v>
       </c>
       <c r="D132" s="4">
         <f t="shared" si="1"/>
-        <v>0.6666666667</v>
+        <v>0</v>
       </c>
       <c r="E132" s="5" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="133" ht="22.5" customHeight="1">
-      <c r="A133" s="10"/>
-      <c r="B133" s="10"/>
-      <c r="C133" s="3"/>
-      <c r="D133" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E133" s="11"/>
+      <c r="A133" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C133" s="3">
+        <v>8.81529680365E10</v>
+      </c>
+      <c r="D133" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E133" s="5" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="134" ht="22.5" customHeight="1">
-      <c r="A134" s="10"/>
-      <c r="B134" s="10"/>
-      <c r="C134" s="8"/>
-      <c r="D134" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E134" s="11"/>
+      <c r="A134" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C134" s="3">
+        <v>2.39E11</v>
+      </c>
+      <c r="D134" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E134" s="9" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="135" ht="22.5" customHeight="1">
-      <c r="A135" s="10"/>
-      <c r="B135" s="10"/>
-      <c r="C135" s="8"/>
-      <c r="D135" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E135" s="11"/>
+      <c r="A135" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C135" s="3">
+        <v>3.2552635E12</v>
+      </c>
+      <c r="D135" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E135" s="5" t="s">
+        <v>270</v>
+      </c>
     </row>
     <row r="136" ht="22.5" customHeight="1">
-      <c r="A136" s="10"/>
-      <c r="B136" s="10"/>
-      <c r="C136" s="8"/>
-      <c r="D136" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E136" s="11"/>
+      <c r="A136" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C136" s="8">
+        <f>3*10^14</f>
+        <v>300000000000000</v>
+      </c>
+      <c r="D136" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E136" s="5" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="137" ht="22.5" customHeight="1">
-      <c r="A137" s="10"/>
-      <c r="B137" s="10"/>
-      <c r="C137" s="8"/>
-      <c r="D137" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E137" s="11"/>
+      <c r="A137" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C137" s="3">
+        <v>1.4285714E15</v>
+      </c>
+      <c r="D137" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E137" s="5" t="s">
+        <v>274</v>
+      </c>
     </row>
     <row r="138" ht="22.5" customHeight="1">
       <c r="A138" s="10"/>
@@ -12518,28 +12588,28 @@
     <hyperlink r:id="rId2" ref="E3"/>
     <hyperlink r:id="rId3" ref="E4"/>
     <hyperlink r:id="rId4" ref="E5"/>
-    <hyperlink r:id="rId5" location=":~:text=a%20major%20league,inches%20in%20circumference." ref="E6"/>
+    <hyperlink r:id="rId5" ref="E6"/>
     <hyperlink r:id="rId6" ref="E7"/>
     <hyperlink r:id="rId7" ref="E8"/>
     <hyperlink r:id="rId8" ref="E9"/>
-    <hyperlink r:id="rId9" location=":~:text=Weight%3A%2055%20Tons," ref="E10"/>
+    <hyperlink r:id="rId9" ref="E10"/>
     <hyperlink r:id="rId10" ref="E11"/>
     <hyperlink r:id="rId11" ref="E12"/>
     <hyperlink r:id="rId12" ref="E13"/>
     <hyperlink r:id="rId13" ref="E14"/>
     <hyperlink r:id="rId14" ref="E15"/>
-    <hyperlink r:id="rId15" ref="E16"/>
-    <hyperlink r:id="rId16" location="c3" ref="E17"/>
+    <hyperlink r:id="rId15" location=":~:text=a%20major%20league,inches%20in%20circumference." ref="E16"/>
+    <hyperlink r:id="rId16" ref="E17"/>
     <hyperlink r:id="rId17" ref="E18"/>
     <hyperlink r:id="rId18" ref="E19"/>
-    <hyperlink r:id="rId19" ref="E20"/>
+    <hyperlink r:id="rId19" location=":~:text=Weight%3A%2055%20Tons," ref="E20"/>
     <hyperlink r:id="rId20" ref="E21"/>
     <hyperlink r:id="rId21" ref="E22"/>
     <hyperlink r:id="rId22" ref="E23"/>
     <hyperlink r:id="rId23" ref="E24"/>
     <hyperlink r:id="rId24" ref="E25"/>
     <hyperlink r:id="rId25" ref="E26"/>
-    <hyperlink r:id="rId26" ref="E27"/>
+    <hyperlink r:id="rId26" location="c3" ref="E27"/>
     <hyperlink r:id="rId27" ref="E28"/>
     <hyperlink r:id="rId28" ref="E29"/>
     <hyperlink r:id="rId29" ref="E30"/>
@@ -12559,7 +12629,7 @@
     <hyperlink r:id="rId43" ref="E44"/>
     <hyperlink r:id="rId44" ref="E45"/>
     <hyperlink r:id="rId45" ref="E46"/>
-    <hyperlink r:id="rId46" location="gsc.tab=0" ref="E47"/>
+    <hyperlink r:id="rId46" ref="E47"/>
     <hyperlink r:id="rId47" ref="E48"/>
     <hyperlink r:id="rId48" ref="E49"/>
     <hyperlink r:id="rId49" ref="E50"/>
@@ -12569,7 +12639,7 @@
     <hyperlink r:id="rId53" ref="E54"/>
     <hyperlink r:id="rId54" ref="E55"/>
     <hyperlink r:id="rId55" ref="E56"/>
-    <hyperlink r:id="rId56" ref="E57"/>
+    <hyperlink r:id="rId56" location="gsc.tab=0" ref="E57"/>
     <hyperlink r:id="rId57" ref="E58"/>
     <hyperlink r:id="rId58" ref="E59"/>
     <hyperlink r:id="rId59" ref="E60"/>
@@ -12577,7 +12647,7 @@
     <hyperlink r:id="rId61" ref="E62"/>
     <hyperlink r:id="rId62" ref="E63"/>
     <hyperlink r:id="rId63" ref="E64"/>
-    <hyperlink r:id="rId64" location="section=Computed-Properties" ref="E65"/>
+    <hyperlink r:id="rId64" ref="E65"/>
     <hyperlink r:id="rId65" ref="E66"/>
     <hyperlink r:id="rId66" ref="E67"/>
     <hyperlink r:id="rId67" ref="E68"/>
@@ -12587,37 +12657,37 @@
     <hyperlink r:id="rId71" ref="E72"/>
     <hyperlink r:id="rId72" ref="E73"/>
     <hyperlink r:id="rId73" ref="E74"/>
-    <hyperlink r:id="rId74" ref="E75"/>
+    <hyperlink r:id="rId74" location="section=Computed-Properties" ref="E75"/>
     <hyperlink r:id="rId75" ref="E76"/>
     <hyperlink r:id="rId76" ref="E77"/>
     <hyperlink r:id="rId77" ref="E78"/>
     <hyperlink r:id="rId78" ref="E79"/>
     <hyperlink r:id="rId79" ref="E80"/>
     <hyperlink r:id="rId80" ref="E81"/>
-    <hyperlink r:id="rId81" location="12252" ref="E82"/>
+    <hyperlink r:id="rId81" ref="E82"/>
     <hyperlink r:id="rId82" ref="E83"/>
     <hyperlink r:id="rId83" ref="E84"/>
     <hyperlink r:id="rId84" ref="E85"/>
     <hyperlink r:id="rId85" ref="E86"/>
     <hyperlink r:id="rId86" ref="E87"/>
     <hyperlink r:id="rId87" ref="E88"/>
-    <hyperlink r:id="rId88" location="Nfaq4.4.3.3" ref="E89"/>
-    <hyperlink r:id="rId89" location="Nfaq4.4.3.3" ref="E90"/>
+    <hyperlink r:id="rId88" ref="E89"/>
+    <hyperlink r:id="rId89" ref="E90"/>
     <hyperlink r:id="rId90" ref="E91"/>
     <hyperlink r:id="rId91" ref="E92"/>
     <hyperlink r:id="rId92" ref="E93"/>
     <hyperlink r:id="rId93" ref="E94"/>
     <hyperlink r:id="rId94" ref="E95"/>
     <hyperlink r:id="rId95" ref="E96"/>
-    <hyperlink r:id="rId96" ref="E97"/>
+    <hyperlink r:id="rId96" location="12252" ref="E97"/>
     <hyperlink r:id="rId97" ref="E98"/>
     <hyperlink r:id="rId98" ref="E99"/>
     <hyperlink r:id="rId99" ref="E100"/>
     <hyperlink r:id="rId100" ref="E101"/>
     <hyperlink r:id="rId101" ref="E102"/>
     <hyperlink r:id="rId102" ref="E103"/>
-    <hyperlink r:id="rId103" ref="E104"/>
-    <hyperlink r:id="rId104" ref="E105"/>
+    <hyperlink r:id="rId103" location="Nfaq4.4.3.3" ref="E104"/>
+    <hyperlink r:id="rId104" location="Nfaq4.4.3.3" ref="E105"/>
     <hyperlink r:id="rId105" ref="E106"/>
     <hyperlink r:id="rId106" ref="E107"/>
     <hyperlink r:id="rId107" ref="E108"/>
@@ -12645,10 +12715,15 @@
     <hyperlink r:id="rId129" ref="E130"/>
     <hyperlink r:id="rId130" ref="E131"/>
     <hyperlink r:id="rId131" ref="E132"/>
+    <hyperlink r:id="rId132" ref="E133"/>
+    <hyperlink r:id="rId133" ref="E134"/>
+    <hyperlink r:id="rId134" ref="E135"/>
+    <hyperlink r:id="rId135" ref="E136"/>
+    <hyperlink r:id="rId136" ref="E137"/>
   </hyperlinks>
-  <drawing r:id="rId132"/>
+  <drawing r:id="rId137"/>
   <tableParts count="1">
-    <tablePart r:id="rId134"/>
+    <tablePart r:id="rId139"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>